<commit_message>
Actualización automatizada de usuarios.xlsx
</commit_message>
<xml_diff>
--- a/usuarios.xlsx
+++ b/usuarios.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="9">
   <si>
     <t>Nombre</t>
   </si>
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t>Mario oaiza</t>
+  </si>
+  <si>
+    <t>Mario Loaiza</t>
   </si>
   <si>
     <t>mario.loaiza@cablemovil.com.co</t>
@@ -369,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -391,13 +394,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -405,13 +408,27 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C4" t="s">
         <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>